<commit_message>
Added final permutation testing script
</commit_message>
<xml_diff>
--- a/data/L3/Supplemental Tables.xlsx
+++ b/data/L3/Supplemental Tables.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eagar\Dropbox\IBEEM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eagar\Dropbox\IBEEM\conspecific_density_dependence\data\L3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC419893-3E2A-4F89-88F1-782634891BE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FFC9167-F4CB-45F7-9EDD-970950308CD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -437,6 +437,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F122"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">

</xml_diff>